<commit_message>
Đồng bộ hai website theo app bản 237 (KHGD Tiếng Việt 1 tuần 1 chia 2/2/6/2 theo SGV)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLmY8gmbc3bt5a6aV9Q81U
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/KHDH ca khoi - Lop 1.xlsx
+++ b/assets/docs/lop1/KHDH ca khoi - Lop 1.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Âm nhạc" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mĩ thuật" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giáo dục thể chất" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoạt động trải nghiệm" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiếng Anh" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoạt động trải nghiệm" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,12 +555,12 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>3 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>1 – 3</t>
+          <t>1 – 2</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -589,12 +590,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>3 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>4 – 6</t>
+          <t>3 – 4</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -619,17 +620,17 @@
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Làm quen với các nét viết cơ bản, các chữ số, dấu thanh và bảng chữ cái</t>
+          <t>Làm quen với các nét cơ bản, các chữ số, bảng chữ cái và dấu thanh</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>3 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>7 – 9</t>
+          <t>5 – 10</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -659,12 +660,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>3 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>10 – 12</t>
+          <t>11 – 12</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -13668,7 +13669,7 @@
       <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Học hát: Vào rừng hoa (Việt Anh)</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Thường thức âm nhạc: Âm thanh kì diệu; Học hát: Vào rừng hoa (Việt Anh)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -13702,7 +13703,7 @@
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Thường thức âm nhạc: Câu chuyện "Âm thanh kì diệu"</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Đọc nhạc: Bậc thang Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -13717,7 +13718,8 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS nghe các đoạn âm thanh GV mở từ học liệu số và nói được đó là tiếng gì.</t>
+          <t>Năng lực số 3.1 CB1a: HS cùng GV tạo bản ghi âm đoạn đọc to – nhỏ của lớp và nghe lại.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -13770,7 +13772,7 @@
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 1: Âm thanh kì diệu — Vận dụng – Sáng tạo: To – Nhỏ</t>
+          <t>Chủ đề 1: Âm thanh kì diệu — Ôn bài hát Vào rừng hoa; Ôn đọc nhạc: Bậc thang Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -13785,7 +13787,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.1 CB1a: HS cùng GV tạo bản ghi âm đoạn đọc to – nhỏ của lớp và nghe lại.
+          <t>Năng lực số 1.1 CB1a: HS nhìn dòng nhạc Đô – Rê – Mi trên màn hình, nghe tiếng đàn và chỉ ra nốt được đọc to hơn.
 KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
@@ -13805,7 +13807,7 @@
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Học hát: Tổ quốc ta (Mộng Lân)</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Học hát: Tổ quốc ta (Mộng Lân); Vận dụng – Sáng tạo: Cao – Thấp</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -13875,7 +13877,7 @@
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Nhạc cụ: Gõ đệm trống con cho bài Tổ quốc ta; Nghe nhạc: Quốc ca (Văn Cao)</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Nghe nhạc: Quốc ca (Văn Cao); Nhạc cụ: Trống con</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -13910,7 +13912,7 @@
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 2: Việt Nam yêu thương — Vận dụng – Sáng tạo: Cao – Thấp</t>
+          <t>Chủ đề 2: Việt Nam yêu thương — Ôn bài hát Tổ quốc ta; Vận dụng – Sáng tạo: Cao – Thấp</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -13925,7 +13927,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS nghe âm thanh GV mở từ học liệu số và nói được âm nào cao, âm nào thấp.
+          <t>Năng lực số 1.1 CB1a: HS nghe tiếng kèn tu-ba, sáo pic-cô-lô GV mở từ học liệu số và nói được âm nào cao, âm nào thấp.
 QPAN: Chọn bài hát ca ngợi quê hương, đất nước, hoà bình; liên hệ hình ảnh chú bộ đội Quân đội nhân dân, chú công an Công an nhân dân và di tích lịch sử ở địa phương.</t>
         </is>
       </c>
@@ -13945,7 +13947,7 @@
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 3: Mái trường thân yêu — Học hát: Lớp Một thân yêu (Bùi Anh Tôn)</t>
+          <t>Chủ đề 3: Mái trường thân yêu — Học hát: Lớp Một thân yêu (Bùi Anh Tôn); Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -13960,7 +13962,8 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát Lớp Một thân yêu cùng tên tác giả Bùi Anh Tôn.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát Lớp Một thân yêu cùng tên tác giả Bùi Anh Tôn.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14047,7 +14050,7 @@
       <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 3: Mái trường thân yêu — Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
+          <t>Chủ đề 3: Mái trường thân yêu — Ôn bài hát Lớp Một thân yêu; Ôn đọc nhạc: Ban nhạc Đô – Rê – Mi; Vận dụng – Sáng tạo: To – Nhỏ, Cao – Thấp</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -14252,7 +14255,7 @@
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Học hát: Xúc xắc xúc xẻ (Nhạc: Nguyễn Ngọc Thiện, lời: phỏng theo đồng dao)</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Học hát: Xúc xắc xúc xẻ (Nhạc: Nguyễn Ngọc Thiện, lời: phỏng theo đồng dao); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -14267,7 +14270,8 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả phần nhạc và nguồn lời ca phỏng theo đồng dao.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả phần nhạc và nguồn lời ca phỏng theo đồng dao.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14320,7 +14324,7 @@
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Thường thức âm nhạc: Nhạc sĩ Mô-da (Câu chuyện "Thần đồng âm nhạc Mô-da"); Nghe nhạc: Khát vọng mùa xuân</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Ôn đọc nhạc: Những người bạn của Đô – Rê – Mi; Thường thức âm nhạc: Nhạc sĩ Vôn-gang A-ma-đớt Mô-da (nghe bài hát Khát vọng mùa xuân); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -14335,7 +14339,8 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe GV giới thiệu và nói được tên nhạc sĩ Mô-da, tên bản nhạc vừa nghe.</t>
+          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe GV giới thiệu và nói được tên nhạc sĩ Mô-da, tên bài hát Khát vọng mùa xuân.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14354,7 +14359,7 @@
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 5: Nhịp điệu mùa xuân — Vận dụng – Sáng tạo: Dài – Ngắn</t>
+          <t>Chủ đề 5: Nhịp điệu mùa xuân — Ôn bài hát Xúc xắc xúc xẻ; Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -14389,7 +14394,7 @@
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Học hát: Gà gáy (Dân ca Cống Khao, lời mới: Huy Trân)</t>
+          <t>Chủ đề 6: Về miền dân ca — Học hát: Gà gáy (Dân ca Cống Khao, lời mới: Huy Trân); Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -14404,7 +14409,8 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được bài Gà gáy là dân ca Cống Khao và người viết lời mới là Huy Trân.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được bài Gà gáy là dân ca Cống Khao và người viết lời mới là Huy Trân.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14423,7 +14429,7 @@
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Thường thức âm nhạc: "Câu chuyện về thanh phách"</t>
+          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Nhạc cụ: Thanh phách</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -14438,7 +14444,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe âm thanh trên màn hình và nói đúng tên nhạc cụ thanh phách.</t>
+          <t>Năng lực số 3.1 CB1a: HS cùng GV ghi âm phần cả lớp hát Gà gáy kết hợp gõ thanh phách và nghe lại để nhận xét tiếng phách đã đều chưa.</t>
         </is>
       </c>
     </row>
@@ -14457,7 +14463,7 @@
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Nhạc cụ: Thanh phách; Nghe nhạc: Lí cây bông (Dân ca Nam Bộ)</t>
+          <t>Chủ đề 6: Về miền dân ca — Thường thức âm nhạc: Câu chuyện về thanh phách; Vận dụng – Sáng tạo: Dài – Ngắn</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -14472,7 +14478,8 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 4.1 CB1a: HS ngồi đúng khoảng cách với màn hình, nghe loa vừa đủ khi xem, nghe bài Lí cây bông.</t>
+          <t>Năng lực số 1.1 CB1a: HS xem hình, nghe âm thanh trên màn hình và nói đúng tên nhạc cụ thanh phách.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14491,7 +14498,7 @@
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 6: Về miền dân ca — Vận dụng – Sáng tạo: Dài – Ngắn</t>
+          <t>Chủ đề 6: Về miền dân ca — Ôn bài hát Gà gáy; Nghe nhạc: Lí cây bông (Dân ca Nam Bộ)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -14506,8 +14513,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 2.1 CB1a: HS nói lời chào buổi sáng để GV ghi lại thành lời nhắn gửi bạn lớp bên.
-KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
+          <t>Năng lực số 4.1 CB1a: HS ngồi đúng khoảng cách với màn hình, nghe loa vừa đủ khi xem, nghe bài Lí cây bông.</t>
         </is>
       </c>
     </row>
@@ -14526,7 +14532,7 @@
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 7: Gia đình — Học hát: Cây gia đình (Nhạc: Quỳnh Hợp, lời thơ: Nguyễn Thị Mai)</t>
+          <t>Chủ đề 7: Gia đình — Học hát: Cây gia đình (Nhạc: Quỳnh Hợp, lời thơ: Nguyễn Thị Mai); Vận dụng – Sáng tạo: Góc âm nhạc</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -14541,7 +14547,8 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả nhạc và tác giả lời thơ.</t>
+          <t>Năng lực số 3.3 CB1a: HS nói được tên bài hát cùng tên tác giả nhạc và tác giả lời thơ.
+KNS: KN tự tin biểu diễn trước tập thể và phối hợp cùng nhóm.</t>
         </is>
       </c>
     </row>
@@ -14628,7 +14635,7 @@
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 7: Gia đình — Vận dụng – Sáng tạo: Góc âm nhạc</t>
+          <t>Chủ đề 7: Gia đình — Vận dụng – Sáng tạo: Góc âm nhạc; Ôn bài hát Cây gia đình</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -14697,7 +14704,7 @@
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Chủ đề 8: Vui đón hè — Ôn bài hát Ngôi sao lấp lánh; Nhạc cụ: Trai-en-gô</t>
+          <t>Chủ đề 8: Vui đón hè — Nhạc cụ: Trai-en-gô (triangle); Ôn bài hát Ngôi sao lấp lánh</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -18431,6 +18438,1363 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KẾ HOẠCH GIÁO DỤC MÔN TIẾNG ANH — LỚP 1 · NĂM HỌC 2026-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cách dùng: giữ nguyên dòng tên cột và thứ tự cột · mỗi tiết một dòng · ô Tuần/Chủ đề/Tên bài để trống nghĩa là giống dòng trên · sửa xong lưu lại rồi vào Bút Xanh bấm "Nhập KHGD của tôi".</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tuần</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Chủ đề/Mạch nội dung</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Tên bài</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Phân môn / Hoạt động</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Nội dung/Tên bài học</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Thời lượng</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Tiết KH</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Nội dung điều chỉnh, bổ sung</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Me and my friends</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Unit 1: In the school playground</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Unit 1: In the school playground – Lesson 1 (1, 2) &amp; Lesson 2 (3, 4, 5)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 1.3.CB1a: Guide pupils to access and open the lesson audio files on a safe digital learning resources website.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Me and my friends</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Unit 1: In the school playground</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Unit 1: In the school playground – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Unit 2: In the dining room</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Unit 2: In the dining room – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Unit 2: In the dining room</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Unit 2: In the dining room – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 3.1.CB1a: Practise drawing a simple birthday cake in Paint
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Fun time 1</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Me and the world around</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Unit 3: At the street market</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Unit 3: At the street market – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 1.1.CB1b: Search safely for pictures of a country market
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Me and my friends</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Unit 3: At the street market</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Unit 3: At the street market – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.C1.3: How an AI camera scans images and recognises circles and squares in real life.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Unit 4: In the bedroom</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Unit 4: In the bedroom – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Unit 4: In the bedroom</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Unit 4: In the bedroom – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Unit 5: At the fish and chip shop</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Unit 5: At the fish and chip shop – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.C1.1: Recognise the AI system in automatic ordering machines that quickly identifies fish dishes.
+Ethics: Know how to say "Thank you" when receiving food from parents or staff.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Unit 5: At the fish and chip shop</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Unit 5: At the fish and chip shop – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.D1.1: For a robot to know the types of milk, pupils need to show the machine pictures of strawberry milk and plain milk cartons so that it does not learn wrongly.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Unit 6: In the classroom</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Unit 6: In the classroom – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.C1.1: Recognise AI in the smart interactive board that helps the teacher practise writing the letter Pp, pen, pencil.
+Digital competence 4.1.CB1a: Turn off the computer at the end of the lesson to protect the device.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Unit 6: In the classroom</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Unit 6: In the classroom – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.A1.1: Discussion: Humans decide to use pencils to draw creative pictures; AI only follows commands.
+Digital competence 3.1.CB1a: Practise drawing a classroom object (a rectangle) on the computer.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Fun time 2</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.C1.1: Compare how fast pupils find words with how fast AI scans data to find the answer in an instant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Unit 7: In the garden</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Unit 7: In the garden – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.C1.1: Recognise smart (AI) devices that automatically water the garden when the soil is dry.
+Ethics: Love nature and protect green trees.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Unit 7: In the garden</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Unit 7: In the garden – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Me and my family</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Unit 8: In the park</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Unit 8: In the park – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Semester I Test &amp; Feedback – Self-check</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Me and the world around</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Unit 9: In the shop</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Unit 9: In the shop – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Me and the world around</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Unit 9: In the shop</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Unit 9: In the shop – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Me and the world around</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Unit 10: At the zoo</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Unit 10: At the zoo – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 1.1.CB1b: Search the Internet for videos of monkey sounds under the teacher's safe guidance.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Me and the world around</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Unit 10: At the zoo</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Unit 10: At the zoo – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>AI 1.A1.1: Discussion: Humans decide what to feed animals; AI can only suggest menus based on available data.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Fun time 3</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Me and my friends</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Unit 11: At the bus stop</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Unit 11: At the bus stop – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 4.3.CB1a: Health risk warning: Do not walk while looking at a phone, so as to stay safe in the sun.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Me and my friends</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Unit 11: At the bus stop</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Unit 11: At the bus stop – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Unit 12: At the lake</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Unit 12: At the lake – Lesson 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 3.1.CB1a: Practise drawing a simple digital leaf or lemon (lemons) on the computer.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Unit 12: At the lake</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Unit 12: At the lake – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Unit 13: In the school canteen</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Unit 13: In the school canteen – Lesson 1, 2</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Unit 13: In the school canteen</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Unit 13: In the school canteen – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Unit 14: In the toy shop</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Unit 14: In the toy shop – Lesson 1, 2</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 4.2.CB1b: Information security: Do not share photos of expensive gifts online, so that bad people cannot take advantage of them.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Fun time 4</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 3.3.CB1a: Respect copyright: Write your name on your drawing before submitting it to the teacher on the interactive board.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Unit 15: At the football match</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Unit 15: At the football match – Lesson 1, 2</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Me and my school</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Unit 15: At the football match</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Unit 15: At the football match – Lesson 3</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Unit 16: At home</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Unit 16: At home – Lesson 1, 2</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Digital competence 1.3.CB1b: Pupils sort pictures of houses into the "My Home" folder on the class computer.
+Life skills: Communication skills: confidently greet others and introduce themselves in simple sentences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Review 4: Self-check</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>1 tiết</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>